<commit_message>
Data Driven - Multiple data - Column constant
</commit_message>
<xml_diff>
--- a/Data Driven Testing/multipledata.xlsx
+++ b/Data Driven Testing/multipledata.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\visual Studio Code WorkSpace\Playwright_B1\Data Driven Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D50EBD-3CAE-406A-AAC3-3D4E764B8496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D974948-C8AE-4E88-9626-B324A767C09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>Jonny</t>
   </si>
@@ -37,6 +38,15 @@
   </si>
   <si>
     <t>Male</t>
+  </si>
+  <si>
+    <t>Raya</t>
+  </si>
+  <si>
+    <t>Karur</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
 </sst>
 </file>
@@ -377,4 +387,39 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD9B5AC4-381F-4CD9-B572-1F90C7937BE8}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Data Driven|Excel|Fetching auto suggessions
</commit_message>
<xml_diff>
--- a/Data Driven Testing/multipledata.xlsx
+++ b/Data Driven Testing/multipledata.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Sheet2" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sheet3" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>Jonny</t>
   </si>
@@ -36,6 +37,36 @@
   </si>
   <si>
     <t>Female</t>
+  </si>
+  <si>
+    <t>laptop under 35000</t>
+  </si>
+  <si>
+    <t>laptop stand metal</t>
+  </si>
+  <si>
+    <t>laptop under 50k</t>
+  </si>
+  <si>
+    <t>laptop under 50k+</t>
+  </si>
+  <si>
+    <t>laptop for gaming</t>
+  </si>
+  <si>
+    <t>laptop under 20000 price</t>
+  </si>
+  <si>
+    <t>laptop bags for men office use</t>
+  </si>
+  <si>
+    <t>laptop bag for man</t>
+  </si>
+  <si>
+    <t>laptop table on bed</t>
+  </si>
+  <si>
+    <t>laptop cleaner kit</t>
   </si>
 </sst>
 </file>
@@ -411,4 +442,65 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>